<commit_message>
warm start for obj func added
</commit_message>
<xml_diff>
--- a/data/fall2425_course_info - Copy.xlsx
+++ b/data/fall2425_course_info - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berkercin\Desktop\Projects\Scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2DDAB3-8307-48B1-B1A7-3681068225B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCFD0E4-7F4E-46BF-A40F-5B216A0069F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>MAK 101</t>
   </si>
   <si>
-    <t>Elektrik-Elektronik Mühendisliği</t>
-  </si>
-  <si>
     <t>İleri Bilgisayar Programlama</t>
   </si>
   <si>
@@ -125,9 +122,6 @@
     <t>İNM 453</t>
   </si>
   <si>
-    <t>Bilgisayar Mühendisliği  (İngilizce)</t>
-  </si>
-  <si>
     <t>Takım Tezgahları</t>
   </si>
   <si>
@@ -563,9 +557,6 @@
     <t>İNM 471</t>
   </si>
   <si>
-    <t>Elektrik-Elektronik Mühendisliğine Giriş</t>
-  </si>
-  <si>
     <t>EEM 107</t>
   </si>
   <si>
@@ -1284,6 +1275,15 @@
   </si>
   <si>
     <t>ÇEV 303L</t>
+  </si>
+  <si>
+    <t>Bilgisayar Mühendisliği</t>
+  </si>
+  <si>
+    <t>Elektrik Elektronik Mühendisliği</t>
+  </si>
+  <si>
+    <t>Elektrik Elektronik Mühendisliğine Giriş</t>
   </si>
 </sst>
 </file>
@@ -1742,18 +1742,18 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
@@ -1762,7 +1762,7 @@
         <v>154</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="F2" s="2">
         <v>0</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C3" s="3">
         <v>1</v>
@@ -1785,7 +1785,7 @@
         <v>135</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F3" s="3">
         <v>1</v>
@@ -1796,10 +1796,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C4" s="3">
         <v>4</v>
@@ -1808,7 +1808,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F4" s="3">
         <v>0</v>
@@ -1822,7 +1822,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="7">
         <v>3</v>
@@ -1831,7 +1831,7 @@
         <v>118</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="7">
         <v>0</v>
@@ -1842,10 +1842,10 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C6" s="3">
         <v>4</v>
@@ -1854,7 +1854,7 @@
         <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F6" s="3">
         <v>0</v>
@@ -1865,10 +1865,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
@@ -1877,7 +1877,7 @@
         <v>146</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -1888,10 +1888,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C8" s="4">
         <v>2</v>
@@ -1900,7 +1900,7 @@
         <v>107</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="F8" s="4">
         <v>0</v>
@@ -1911,10 +1911,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
@@ -1923,7 +1923,7 @@
         <v>14</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -1934,10 +1934,10 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C10" s="5">
         <v>2</v>
@@ -1946,7 +1946,7 @@
         <v>96</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F10" s="5">
         <v>1</v>
@@ -1957,10 +1957,10 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C11" s="8">
         <v>1</v>
@@ -1969,7 +1969,7 @@
         <v>175</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F11" s="8">
         <v>1</v>
@@ -1980,10 +1980,10 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" s="3">
         <v>2</v>
@@ -1992,7 +1992,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="F12" s="3">
         <v>0</v>
@@ -2003,10 +2003,10 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="C13" s="3">
         <v>4</v>
@@ -2015,7 +2015,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="F13" s="3">
         <v>0</v>
@@ -2026,10 +2026,10 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C14" s="4">
         <v>3</v>
@@ -2038,7 +2038,7 @@
         <v>20</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F14" s="4">
         <v>0</v>
@@ -2049,10 +2049,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C15" s="5">
         <v>3</v>
@@ -2061,7 +2061,7 @@
         <v>129</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F15" s="5">
         <v>0</v>
@@ -2072,10 +2072,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C16" s="5">
         <v>4</v>
@@ -2084,7 +2084,7 @@
         <v>49</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F16" s="5">
         <v>0</v>
@@ -2098,7 +2098,7 @@
         <v>6</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C17" s="7">
         <v>4</v>
@@ -2107,7 +2107,7 @@
         <v>21</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="F17" s="7">
         <v>0</v>
@@ -2118,10 +2118,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C18" s="8">
         <v>1</v>
@@ -2130,7 +2130,7 @@
         <v>214</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F18" s="8">
         <v>0</v>
@@ -2141,10 +2141,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
@@ -2153,7 +2153,7 @@
         <v>65</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F19" s="5">
         <v>0</v>
@@ -2164,10 +2164,10 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C20" s="4">
         <v>2</v>
@@ -2176,7 +2176,7 @@
         <v>26</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="F20" s="4">
         <v>0</v>
@@ -2187,10 +2187,10 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C21" s="8">
         <v>4</v>
@@ -2199,7 +2199,7 @@
         <v>52</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F21" s="8">
         <v>0</v>
@@ -2210,10 +2210,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C22" s="3">
         <v>1</v>
@@ -2222,7 +2222,7 @@
         <v>19</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F22" s="3">
         <v>0</v>
@@ -2233,10 +2233,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C23" s="5">
         <v>4</v>
@@ -2245,7 +2245,7 @@
         <v>21</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F23" s="5">
         <v>0</v>
@@ -2259,7 +2259,7 @@
         <v>5</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C24" s="6">
         <v>3</v>
@@ -2268,7 +2268,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F24" s="6">
         <v>0</v>
@@ -2279,10 +2279,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C25" s="4">
         <v>1</v>
@@ -2291,7 +2291,7 @@
         <v>73</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F25" s="4">
         <v>0</v>
@@ -2302,10 +2302,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C26" s="8">
         <v>4</v>
@@ -2314,7 +2314,7 @@
         <v>93</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F26" s="8">
         <v>0</v>
@@ -2325,10 +2325,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C27" s="5">
         <v>4</v>
@@ -2337,7 +2337,7 @@
         <v>18</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F27" s="5">
         <v>0</v>
@@ -2348,10 +2348,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C28" s="8">
         <v>4</v>
@@ -2360,7 +2360,7 @@
         <v>45</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F28" s="8">
         <v>0</v>
@@ -2371,10 +2371,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>20</v>
       </c>
       <c r="C29" s="3">
         <v>3</v>
@@ -2383,7 +2383,7 @@
         <v>6</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F29" s="3">
         <v>0</v>
@@ -2394,10 +2394,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C30" s="3">
         <v>4</v>
@@ -2406,7 +2406,7 @@
         <v>8</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="F30" s="3">
         <v>0</v>
@@ -2417,10 +2417,10 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C31" s="3">
         <v>2</v>
@@ -2429,7 +2429,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
@@ -2440,10 +2440,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C32" s="2">
         <v>1</v>
@@ -2452,7 +2452,7 @@
         <v>140</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F32" s="2">
         <v>0</v>
@@ -2463,10 +2463,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C33" s="2">
         <v>1</v>
@@ -2475,7 +2475,7 @@
         <v>167</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F33" s="2">
         <v>0</v>
@@ -2486,10 +2486,10 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C34" s="2">
         <v>1</v>
@@ -2498,7 +2498,7 @@
         <v>185</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F34" s="2">
         <v>0</v>
@@ -2509,10 +2509,10 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C35" s="8">
         <v>4</v>
@@ -2521,7 +2521,7 @@
         <v>64</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F35" s="8">
         <v>0</v>
@@ -2532,10 +2532,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C36" s="3">
         <v>4</v>
@@ -2544,7 +2544,7 @@
         <v>12</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="F36" s="3">
         <v>0</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C37" s="5">
         <v>4</v>
@@ -2567,7 +2567,7 @@
         <v>47</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F37" s="5">
         <v>0</v>
@@ -2578,10 +2578,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C38" s="2">
         <v>1</v>
@@ -2590,7 +2590,7 @@
         <v>258</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F38" s="2">
         <v>1</v>
@@ -2601,10 +2601,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C39" s="8">
         <v>2</v>
@@ -2613,7 +2613,7 @@
         <v>137</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F39" s="8">
         <v>0</v>
@@ -2624,10 +2624,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C40" s="8">
         <v>2</v>
@@ -2636,7 +2636,7 @@
         <v>220</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F40" s="8">
         <v>0</v>
@@ -2650,7 +2650,7 @@
         <v>6</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C41" s="7">
         <v>2</v>
@@ -2659,7 +2659,7 @@
         <v>133</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F41" s="7">
         <v>0</v>
@@ -2670,10 +2670,10 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C42" s="3">
         <v>4</v>
@@ -2682,7 +2682,7 @@
         <v>1</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2693,10 +2693,10 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C43" s="4">
         <v>2</v>
@@ -2705,7 +2705,7 @@
         <v>115</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="F43" s="4">
         <v>0</v>
@@ -2716,10 +2716,10 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C44" s="5">
         <v>2</v>
@@ -2728,7 +2728,7 @@
         <v>168</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F44" s="5">
         <v>0</v>
@@ -2739,10 +2739,10 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C45" s="8">
         <v>4</v>
@@ -2751,7 +2751,7 @@
         <v>52</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F45" s="8">
         <v>0</v>
@@ -2762,10 +2762,10 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C46" s="2">
         <v>1</v>
@@ -2774,7 +2774,7 @@
         <v>110</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F46" s="2">
         <v>1</v>
@@ -2785,10 +2785,10 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="C47" s="5">
         <v>2</v>
@@ -2797,7 +2797,7 @@
         <v>129</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
@@ -2811,7 +2811,7 @@
         <v>6</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C48" s="7">
         <v>4</v>
@@ -2820,7 +2820,7 @@
         <v>19</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F48" s="7">
         <v>0</v>
@@ -2831,10 +2831,10 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C49" s="4">
         <v>3</v>
@@ -2843,7 +2843,7 @@
         <v>29</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F49" s="4">
         <v>0</v>
@@ -2854,10 +2854,10 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C50" s="8">
         <v>3</v>
@@ -2866,7 +2866,7 @@
         <v>226</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F50" s="8">
         <v>0</v>
@@ -2877,10 +2877,10 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C51" s="8">
         <v>3</v>
@@ -2889,7 +2889,7 @@
         <v>45</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F51" s="8">
         <v>0</v>
@@ -2900,10 +2900,10 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C52" s="8">
         <v>3</v>
@@ -2912,7 +2912,7 @@
         <v>179</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F52" s="8">
         <v>0</v>
@@ -2923,10 +2923,10 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C53" s="8">
         <v>3</v>
@@ -2935,7 +2935,7 @@
         <v>139</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F53" s="8">
         <v>0</v>
@@ -2946,10 +2946,10 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C54" s="8">
         <v>3</v>
@@ -2958,7 +2958,7 @@
         <v>92</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F54" s="8">
         <v>0</v>
@@ -2969,10 +2969,10 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C55" s="8">
         <v>3</v>
@@ -2981,7 +2981,7 @@
         <v>62</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="F55" s="8">
         <v>0</v>
@@ -2992,10 +2992,10 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>175</v>
+        <v>415</v>
       </c>
       <c r="C56" s="8">
         <v>1</v>
@@ -3004,7 +3004,7 @@
         <v>183</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F56" s="8">
         <v>0</v>
@@ -3015,10 +3015,10 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C57" s="8">
         <v>2</v>
@@ -3027,7 +3027,7 @@
         <v>221</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F57" s="8">
         <v>0</v>
@@ -3038,10 +3038,10 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C58" s="8">
         <v>4</v>
@@ -3050,7 +3050,7 @@
         <v>79</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F58" s="8">
         <v>0</v>
@@ -3061,10 +3061,10 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C59" s="4">
         <v>3</v>
@@ -3073,7 +3073,7 @@
         <v>16</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F59" s="4">
         <v>0</v>
@@ -3084,10 +3084,10 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C60" s="2">
         <v>2</v>
@@ -3096,7 +3096,7 @@
         <v>86</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F60" s="2">
         <v>1</v>
@@ -3107,10 +3107,10 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C61" s="2">
         <v>2</v>
@@ -3119,7 +3119,7 @@
         <v>99</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F61" s="2">
         <v>0</v>
@@ -3130,10 +3130,10 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C62" s="4">
         <v>4</v>
@@ -3142,7 +3142,7 @@
         <v>78</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F62" s="4">
         <v>0</v>
@@ -3153,10 +3153,10 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C63" s="2">
         <v>2</v>
@@ -3165,7 +3165,7 @@
         <v>93</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F63" s="2">
         <v>0</v>
@@ -3176,10 +3176,10 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C64" s="3">
         <v>2</v>
@@ -3188,7 +3188,7 @@
         <v>25</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F64" s="3">
         <v>0</v>
@@ -3202,7 +3202,7 @@
         <v>6</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C65" s="7">
         <v>4</v>
@@ -3211,7 +3211,7 @@
         <v>20</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F65" s="7">
         <v>0</v>
@@ -3222,10 +3222,10 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C66" s="4">
         <v>4</v>
@@ -3234,7 +3234,7 @@
         <v>33</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F66" s="4">
         <v>0</v>
@@ -3245,10 +3245,10 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C67" s="4">
         <v>1</v>
@@ -3257,7 +3257,7 @@
         <v>159</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F67" s="4">
         <v>0</v>
@@ -3271,7 +3271,7 @@
         <v>6</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C68" s="7">
         <v>1</v>
@@ -3280,7 +3280,7 @@
         <v>131</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F68" s="7">
         <v>0</v>
@@ -3291,10 +3291,10 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C69" s="5">
         <v>1</v>
@@ -3303,7 +3303,7 @@
         <v>104</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F69" s="5">
         <v>0</v>
@@ -3314,10 +3314,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C70" s="4">
         <v>2</v>
@@ -3326,7 +3326,7 @@
         <v>81</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F70" s="4">
         <v>0</v>
@@ -3337,10 +3337,10 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C71" s="2">
         <v>2</v>
@@ -3349,7 +3349,7 @@
         <v>132</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F71" s="2">
         <v>0</v>
@@ -3360,10 +3360,10 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C72" s="8">
         <v>4</v>
@@ -3372,7 +3372,7 @@
         <v>26</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F72" s="8">
         <v>0</v>
@@ -3383,10 +3383,10 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C73" s="8">
         <v>1</v>
@@ -3395,7 +3395,7 @@
         <v>198</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F73" s="8">
         <v>0</v>
@@ -3406,10 +3406,10 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C74" s="2">
         <v>2</v>
@@ -3418,7 +3418,7 @@
         <v>110</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="F74" s="2">
         <v>0</v>
@@ -3429,10 +3429,10 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C75" s="3">
         <v>2</v>
@@ -3441,7 +3441,7 @@
         <v>9</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F75" s="3">
         <v>0</v>
@@ -3452,10 +3452,10 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C76" s="2">
         <v>2</v>
@@ -3464,7 +3464,7 @@
         <v>60</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F76" s="2">
         <v>0</v>
@@ -3475,10 +3475,10 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C77" s="2">
         <v>3</v>
@@ -3487,7 +3487,7 @@
         <v>119</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F77" s="2">
         <v>0</v>
@@ -3498,10 +3498,10 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C78" s="2">
         <v>3</v>
@@ -3510,7 +3510,7 @@
         <v>99</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="F78" s="2">
         <v>0</v>
@@ -3524,7 +3524,7 @@
         <v>6</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C79" s="7">
         <v>1</v>
@@ -3533,7 +3533,7 @@
         <v>119</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F79" s="7">
         <v>0</v>
@@ -3544,10 +3544,10 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C80" s="5">
         <v>1</v>
@@ -3556,7 +3556,7 @@
         <v>65</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F80" s="5">
         <v>0</v>
@@ -3567,10 +3567,10 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C81" s="4">
         <v>1</v>
@@ -3579,7 +3579,7 @@
         <v>84</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="F81" s="4">
         <v>0</v>
@@ -3590,10 +3590,10 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C82" s="4">
         <v>2</v>
@@ -3602,7 +3602,7 @@
         <v>97</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F82" s="4">
         <v>0</v>
@@ -3613,10 +3613,10 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C83" s="3">
         <v>2</v>
@@ -3625,7 +3625,7 @@
         <v>26</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F83" s="3">
         <v>0</v>
@@ -3636,10 +3636,10 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C84" s="4">
         <v>3</v>
@@ -3648,7 +3648,7 @@
         <v>76</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="F84" s="4">
         <v>0</v>
@@ -3659,10 +3659,10 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C85" s="4">
         <v>4</v>
@@ -3671,7 +3671,7 @@
         <v>72</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F85" s="4">
         <v>0</v>
@@ -3682,10 +3682,10 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C86" s="4">
         <v>3</v>
@@ -3694,7 +3694,7 @@
         <v>32</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F86" s="4">
         <v>0</v>
@@ -3705,10 +3705,10 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C87" s="4">
         <v>4</v>
@@ -3717,7 +3717,7 @@
         <v>63</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F87" s="4">
         <v>0</v>
@@ -3728,10 +3728,10 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C88" s="4">
         <v>2</v>
@@ -3740,7 +3740,7 @@
         <v>100</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F88" s="4">
         <v>0</v>
@@ -3751,10 +3751,10 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C89" s="4">
         <v>3</v>
@@ -3763,7 +3763,7 @@
         <v>35</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F89" s="4">
         <v>0</v>
@@ -3774,10 +3774,10 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C90" s="4">
         <v>3</v>
@@ -3786,7 +3786,7 @@
         <v>29</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F90" s="4">
         <v>0</v>
@@ -3797,10 +3797,10 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C91" s="4">
         <v>1</v>
@@ -3809,7 +3809,7 @@
         <v>76</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="F91" s="4">
         <v>0</v>
@@ -3820,10 +3820,10 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C92" s="4">
         <v>3</v>
@@ -3832,7 +3832,7 @@
         <v>90</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F92" s="4">
         <v>0</v>
@@ -3843,10 +3843,10 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B93" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="C93" s="4">
         <v>2</v>
@@ -3855,7 +3855,7 @@
         <v>45</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F93" s="4">
         <v>0</v>
@@ -3869,7 +3869,7 @@
         <v>6</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C94" s="7">
         <v>3</v>
@@ -3878,7 +3878,7 @@
         <v>24</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F94" s="7">
         <v>0</v>
@@ -3889,10 +3889,10 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C95" s="5">
         <v>3</v>
@@ -3901,7 +3901,7 @@
         <v>110</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F95" s="5">
         <v>0</v>
@@ -3915,7 +3915,7 @@
         <v>6</v>
       </c>
       <c r="B96" s="7" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C96" s="7">
         <v>4</v>
@@ -3924,7 +3924,7 @@
         <v>15</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="F96" s="7">
         <v>0</v>
@@ -3935,10 +3935,10 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C97" s="5">
         <v>3</v>
@@ -3947,7 +3947,7 @@
         <v>84</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="F97" s="5">
         <v>0</v>
@@ -3961,7 +3961,7 @@
         <v>6</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C98" s="7">
         <v>4</v>
@@ -3970,7 +3970,7 @@
         <v>20</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F98" s="7">
         <v>0</v>
@@ -3981,10 +3981,10 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="B99" s="8" t="s">
         <v>9</v>
-      </c>
-      <c r="B99" s="8" t="s">
-        <v>10</v>
       </c>
       <c r="C99" s="8">
         <v>3</v>
@@ -3993,7 +3993,7 @@
         <v>34</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F99" s="8">
         <v>0</v>
@@ -4007,7 +4007,7 @@
         <v>6</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C100" s="7">
         <v>3</v>
@@ -4016,7 +4016,7 @@
         <v>24</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F100" s="7">
         <v>0</v>
@@ -4027,10 +4027,10 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C101" s="8">
         <v>4</v>
@@ -4039,7 +4039,7 @@
         <v>10</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F101" s="8">
         <v>0</v>
@@ -4053,7 +4053,7 @@
         <v>6</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C102" s="7">
         <v>3</v>
@@ -4062,7 +4062,7 @@
         <v>105</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F102" s="7">
         <v>0</v>
@@ -4073,10 +4073,10 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C103" s="4">
         <v>1</v>
@@ -4085,7 +4085,7 @@
         <v>240</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F103" s="4">
         <v>1</v>
@@ -4096,10 +4096,10 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C104" s="5">
         <v>4</v>
@@ -4108,7 +4108,7 @@
         <v>20</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F104" s="5">
         <v>0</v>
@@ -4119,10 +4119,10 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C105" s="5">
         <v>1</v>
@@ -4131,7 +4131,7 @@
         <v>66</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="F105" s="5">
         <v>0</v>
@@ -4142,10 +4142,10 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="C106" s="2">
         <v>1</v>
@@ -4154,7 +4154,7 @@
         <v>8</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="F106" s="2">
         <v>0</v>
@@ -4165,10 +4165,10 @@
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C107" s="2">
         <v>3</v>
@@ -4177,7 +4177,7 @@
         <v>83</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F107" s="2">
         <v>0</v>
@@ -4188,10 +4188,10 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C108" s="8">
         <v>3</v>
@@ -4200,7 +4200,7 @@
         <v>121</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="F108" s="8">
         <v>0</v>
@@ -4211,10 +4211,10 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C109" s="3">
         <v>1</v>
@@ -4223,7 +4223,7 @@
         <v>23</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F109" s="3">
         <v>0</v>
@@ -4234,10 +4234,10 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C110" s="2">
         <v>3</v>
@@ -4246,7 +4246,7 @@
         <v>66</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F110" s="2">
         <v>0</v>
@@ -4257,10 +4257,10 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C111" s="2">
         <v>3</v>
@@ -4269,7 +4269,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F111" s="2">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>5</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C112" s="6">
         <v>4</v>
@@ -4292,7 +4292,7 @@
         <v>8</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F112" s="6">
         <v>0</v>
@@ -4303,10 +4303,10 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C113" s="8">
         <v>4</v>
@@ -4315,7 +4315,7 @@
         <v>59</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="F113" s="8">
         <v>0</v>
@@ -4326,10 +4326,10 @@
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C114" s="4">
         <v>3</v>
@@ -4338,7 +4338,7 @@
         <v>97</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F114" s="4">
         <v>0</v>
@@ -4352,7 +4352,7 @@
         <v>6</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C115" s="7">
         <v>4</v>
@@ -4361,7 +4361,7 @@
         <v>15</v>
       </c>
       <c r="E115" s="7" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="F115" s="7">
         <v>0</v>
@@ -4375,7 +4375,7 @@
         <v>5</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C116" s="6">
         <v>3</v>
@@ -4384,7 +4384,7 @@
         <v>3</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F116" s="6">
         <v>0</v>
@@ -4398,7 +4398,7 @@
         <v>5</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C117" s="6">
         <v>1</v>
@@ -4407,7 +4407,7 @@
         <v>16</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F117" s="6">
         <v>0</v>
@@ -4421,7 +4421,7 @@
         <v>5</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C118" s="6">
         <v>4</v>
@@ -4430,7 +4430,7 @@
         <v>8</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F118" s="6">
         <v>0</v>
@@ -4444,7 +4444,7 @@
         <v>6</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C119" s="7">
         <v>4</v>
@@ -4453,7 +4453,7 @@
         <v>24</v>
       </c>
       <c r="E119" s="7" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="F119" s="7">
         <v>0</v>
@@ -4464,10 +4464,10 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C120" s="5">
         <v>3</v>
@@ -4476,7 +4476,7 @@
         <v>106</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F120" s="5">
         <v>0</v>
@@ -4487,10 +4487,10 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C121" s="8">
         <v>1</v>
@@ -4499,7 +4499,7 @@
         <v>150</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F121" s="8">
         <v>0</v>
@@ -4513,7 +4513,7 @@
         <v>6</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C122" s="7">
         <v>1</v>
@@ -4522,7 +4522,7 @@
         <v>96</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F122" s="7">
         <v>0</v>
@@ -4536,7 +4536,7 @@
         <v>5</v>
       </c>
       <c r="B123" s="6" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C123" s="6">
         <v>1</v>
@@ -4545,7 +4545,7 @@
         <v>14</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F123" s="6">
         <v>0</v>
@@ -4556,10 +4556,10 @@
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C124" s="3">
         <v>1</v>
@@ -4568,7 +4568,7 @@
         <v>31</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F124" s="3">
         <v>0</v>
@@ -4582,7 +4582,7 @@
         <v>5</v>
       </c>
       <c r="B125" s="6" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C125" s="6">
         <v>3</v>
@@ -4591,7 +4591,7 @@
         <v>6</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="F125" s="6">
         <v>0</v>
@@ -4605,7 +4605,7 @@
         <v>6</v>
       </c>
       <c r="B126" s="7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C126" s="7">
         <v>4</v>
@@ -4614,7 +4614,7 @@
         <v>20</v>
       </c>
       <c r="E126" s="7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F126" s="7">
         <v>0</v>
@@ -4625,10 +4625,10 @@
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C127" s="3">
         <v>3</v>
@@ -4637,7 +4637,7 @@
         <v>14</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F127" s="3">
         <v>0</v>
@@ -4651,7 +4651,7 @@
         <v>5</v>
       </c>
       <c r="B128" s="6" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C128" s="6">
         <v>3</v>
@@ -4660,7 +4660,7 @@
         <v>4</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="F128" s="6">
         <v>0</v>
@@ -4674,7 +4674,7 @@
         <v>6</v>
       </c>
       <c r="B129" s="7" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C129" s="7">
         <v>4</v>
@@ -4683,7 +4683,7 @@
         <v>22</v>
       </c>
       <c r="E129" s="7" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F129" s="7">
         <v>0</v>
@@ -4697,7 +4697,7 @@
         <v>5</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C130" s="6">
         <v>2</v>
@@ -4706,7 +4706,7 @@
         <v>9</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F130" s="6">
         <v>0</v>
@@ -4717,10 +4717,10 @@
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C131" s="4">
         <v>3</v>
@@ -4729,7 +4729,7 @@
         <v>103</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="F131" s="4">
         <v>0</v>
@@ -4740,10 +4740,10 @@
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C132" s="4">
         <v>2</v>
@@ -4752,7 +4752,7 @@
         <v>130</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="F132" s="4">
         <v>0</v>
@@ -4766,7 +4766,7 @@
         <v>5</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C133" s="6">
         <v>3</v>
@@ -4775,7 +4775,7 @@
         <v>5</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F133" s="6">
         <v>0</v>
@@ -4789,7 +4789,7 @@
         <v>6</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C134" s="7">
         <v>1</v>
@@ -4798,7 +4798,7 @@
         <v>102</v>
       </c>
       <c r="E134" s="7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F134" s="7">
         <v>0</v>
@@ -4812,7 +4812,7 @@
         <v>6</v>
       </c>
       <c r="B135" s="7" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C135" s="7">
         <v>3</v>
@@ -4821,7 +4821,7 @@
         <v>124</v>
       </c>
       <c r="E135" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F135" s="7">
         <v>0</v>
@@ -4835,7 +4835,7 @@
         <v>6</v>
       </c>
       <c r="B136" s="7" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C136" s="7">
         <v>4</v>
@@ -4844,7 +4844,7 @@
         <v>52</v>
       </c>
       <c r="E136" s="7" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="F136" s="7">
         <v>0</v>
@@ -4855,10 +4855,10 @@
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C137" s="5">
         <v>2</v>
@@ -4867,7 +4867,7 @@
         <v>152</v>
       </c>
       <c r="E137" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F137" s="5">
         <v>0</v>
@@ -4881,7 +4881,7 @@
         <v>6</v>
       </c>
       <c r="B138" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C138" s="7">
         <v>2</v>
@@ -4890,7 +4890,7 @@
         <v>118</v>
       </c>
       <c r="E138" s="7" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F138" s="7">
         <v>0</v>
@@ -4901,10 +4901,10 @@
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C139" s="8">
         <v>2</v>
@@ -4913,7 +4913,7 @@
         <v>182</v>
       </c>
       <c r="E139" s="8" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F139" s="8">
         <v>0</v>
@@ -4924,10 +4924,10 @@
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B140" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C140" s="8">
         <v>2</v>
@@ -4936,7 +4936,7 @@
         <v>132</v>
       </c>
       <c r="E140" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F140" s="8">
         <v>0</v>
@@ -4947,10 +4947,10 @@
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C141" s="5">
         <v>1</v>
@@ -4959,7 +4959,7 @@
         <v>106</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F141" s="5">
         <v>0</v>
@@ -4970,10 +4970,10 @@
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C142" s="4">
         <v>1</v>
@@ -4982,7 +4982,7 @@
         <v>114</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F142" s="4">
         <v>0</v>
@@ -4996,7 +4996,7 @@
         <v>6</v>
       </c>
       <c r="B143" s="7" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C143" s="7">
         <v>1</v>
@@ -5005,7 +5005,7 @@
         <v>140</v>
       </c>
       <c r="E143" s="7" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F143" s="7">
         <v>0</v>
@@ -5016,10 +5016,10 @@
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C144" s="8">
         <v>1</v>
@@ -5028,7 +5028,7 @@
         <v>235</v>
       </c>
       <c r="E144" s="8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F144" s="8">
         <v>0</v>
@@ -5039,10 +5039,10 @@
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C145" s="2">
         <v>3</v>
@@ -5051,7 +5051,7 @@
         <v>9</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F145" s="2">
         <v>0</v>
@@ -5065,7 +5065,7 @@
         <v>6</v>
       </c>
       <c r="B146" s="7" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C146" s="7">
         <v>3</v>
@@ -5074,7 +5074,7 @@
         <v>62</v>
       </c>
       <c r="E146" s="7" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="F146" s="7">
         <v>0</v>
@@ -5085,10 +5085,10 @@
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C147" s="3">
         <v>1</v>
@@ -5097,7 +5097,7 @@
         <v>40</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="F147" s="3">
         <v>0</v>
@@ -5108,10 +5108,10 @@
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C148" s="3">
         <v>3</v>
@@ -5120,7 +5120,7 @@
         <v>9</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="F148" s="3">
         <v>0</v>
@@ -5131,10 +5131,10 @@
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C149" s="4">
         <v>4</v>
@@ -5143,7 +5143,7 @@
         <v>37</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F149" s="4">
         <v>0</v>
@@ -5154,10 +5154,10 @@
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C150" s="4">
         <v>4</v>
@@ -5166,7 +5166,7 @@
         <v>37</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F150" s="4">
         <v>0</v>
@@ -5177,10 +5177,10 @@
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C151" s="2">
         <v>3</v>
@@ -5189,7 +5189,7 @@
         <v>97</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F151" s="2">
         <v>0</v>
@@ -5200,10 +5200,10 @@
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C152" s="2">
         <v>4</v>
@@ -5212,7 +5212,7 @@
         <v>7</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F152" s="2">
         <v>0</v>
@@ -5223,10 +5223,10 @@
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C153" s="4">
         <v>3</v>
@@ -5235,7 +5235,7 @@
         <v>32</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="F153" s="4">
         <v>0</v>
@@ -5246,10 +5246,10 @@
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C154" s="4">
         <v>2</v>
@@ -5258,7 +5258,7 @@
         <v>111</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="F154" s="4">
         <v>0</v>
@@ -5272,7 +5272,7 @@
         <v>5</v>
       </c>
       <c r="B155" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C155" s="6">
         <v>4</v>
@@ -5281,7 +5281,7 @@
         <v>7</v>
       </c>
       <c r="E155" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F155" s="6">
         <v>0</v>
@@ -5292,10 +5292,10 @@
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B156" s="8" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C156" s="8">
         <v>2</v>
@@ -5304,7 +5304,7 @@
         <v>172</v>
       </c>
       <c r="E156" s="8" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F156" s="8">
         <v>0</v>
@@ -5315,10 +5315,10 @@
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B157" s="8" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C157" s="8">
         <v>3</v>
@@ -5327,7 +5327,7 @@
         <v>59</v>
       </c>
       <c r="E157" s="8" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F157" s="8">
         <v>0</v>
@@ -5341,7 +5341,7 @@
         <v>5</v>
       </c>
       <c r="B158" s="6" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C158" s="6">
         <v>2</v>
@@ -5350,7 +5350,7 @@
         <v>2</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F158" s="6">
         <v>0</v>
@@ -5361,10 +5361,10 @@
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C159" s="5">
         <v>2</v>
@@ -5373,7 +5373,7 @@
         <v>64</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F159" s="5">
         <v>0</v>
@@ -5387,7 +5387,7 @@
         <v>6</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C160" s="7">
         <v>2</v>
@@ -5396,7 +5396,7 @@
         <v>123</v>
       </c>
       <c r="E160" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F160" s="7">
         <v>0</v>
@@ -5407,10 +5407,10 @@
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C161" s="2">
         <v>4</v>
@@ -5419,7 +5419,7 @@
         <v>91</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F161" s="2">
         <v>0</v>
@@ -5430,10 +5430,10 @@
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C162" s="2">
         <v>4</v>
@@ -5442,7 +5442,7 @@
         <v>81</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="F162" s="2">
         <v>0</v>
@@ -5453,10 +5453,10 @@
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C163" s="2">
         <v>4</v>
@@ -5465,7 +5465,7 @@
         <v>91</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F163" s="2">
         <v>0</v>
@@ -5476,10 +5476,10 @@
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C164" s="5">
         <v>2</v>
@@ -5488,7 +5488,7 @@
         <v>99</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F164" s="5">
         <v>0</v>
@@ -5502,7 +5502,7 @@
         <v>6</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C165" s="7">
         <v>2</v>
@@ -5511,7 +5511,7 @@
         <v>99</v>
       </c>
       <c r="E165" s="7" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="F165" s="7">
         <v>0</v>
@@ -5522,10 +5522,10 @@
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C166" s="5">
         <v>4</v>
@@ -5534,7 +5534,7 @@
         <v>10</v>
       </c>
       <c r="E166" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F166" s="5">
         <v>0</v>
@@ -5548,7 +5548,7 @@
         <v>6</v>
       </c>
       <c r="B167" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C167" s="7">
         <v>3</v>
@@ -5557,7 +5557,7 @@
         <v>70</v>
       </c>
       <c r="E167" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F167" s="7">
         <v>0</v>
@@ -5568,10 +5568,10 @@
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B168" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C168" s="8">
         <v>4</v>
@@ -5580,7 +5580,7 @@
         <v>69</v>
       </c>
       <c r="E168" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F168" s="8">
         <v>0</v>
@@ -5594,7 +5594,7 @@
         <v>5</v>
       </c>
       <c r="B169" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C169" s="6">
         <v>4</v>
@@ -5603,7 +5603,7 @@
         <v>9</v>
       </c>
       <c r="E169" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F169" s="6">
         <v>0</v>
@@ -5614,10 +5614,10 @@
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C170" s="3">
         <v>4</v>
@@ -5626,7 +5626,7 @@
         <v>17</v>
       </c>
       <c r="E170" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F170" s="3">
         <v>0</v>
@@ -5637,10 +5637,10 @@
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C171" s="2">
         <v>4</v>
@@ -5649,7 +5649,7 @@
         <v>59</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F171" s="2">
         <v>0</v>
@@ -5660,10 +5660,10 @@
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B172" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C172" s="8">
         <v>1</v>
@@ -5672,7 +5672,7 @@
         <v>67</v>
       </c>
       <c r="E172" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F172" s="8">
         <v>1</v>
@@ -5683,10 +5683,10 @@
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C173" s="3">
         <v>3</v>
@@ -5695,7 +5695,7 @@
         <v>14</v>
       </c>
       <c r="E173" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="F173" s="3">
         <v>0</v>
@@ -5706,10 +5706,10 @@
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B174" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C174" s="8">
         <v>1</v>
@@ -5718,7 +5718,7 @@
         <v>142</v>
       </c>
       <c r="E174" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F174" s="8">
         <v>1</v>
@@ -5729,10 +5729,10 @@
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C175" s="2">
         <v>4</v>
@@ -5741,7 +5741,7 @@
         <v>35</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F175" s="2">
         <v>0</v>
@@ -5752,10 +5752,10 @@
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B176" s="8" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C176" s="8">
         <v>4</v>
@@ -5764,7 +5764,7 @@
         <v>64</v>
       </c>
       <c r="E176" s="8" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="F176" s="8">
         <v>0</v>
@@ -5775,10 +5775,10 @@
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C177" s="2">
         <v>4</v>
@@ -5787,7 +5787,7 @@
         <v>56</v>
       </c>
       <c r="E177" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="F177" s="2">
         <v>0</v>
@@ -5798,10 +5798,10 @@
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B178" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C178" s="8">
         <v>2</v>
@@ -5810,7 +5810,7 @@
         <v>183</v>
       </c>
       <c r="E178" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F178" s="8">
         <v>0</v>
@@ -5824,7 +5824,7 @@
         <v>6</v>
       </c>
       <c r="B179" s="7" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C179" s="7">
         <v>4</v>
@@ -5833,7 +5833,7 @@
         <v>19</v>
       </c>
       <c r="E179" s="7" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F179" s="7">
         <v>0</v>
@@ -5847,7 +5847,7 @@
         <v>6</v>
       </c>
       <c r="B180" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C180" s="7">
         <v>4</v>
@@ -5856,7 +5856,7 @@
         <v>31</v>
       </c>
       <c r="E180" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F180" s="7">
         <v>0</v>
@@ -5867,10 +5867,10 @@
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B181" s="5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C181" s="5">
         <v>2</v>
@@ -5879,7 +5879,7 @@
         <v>139</v>
       </c>
       <c r="E181" s="5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F181" s="5">
         <v>0</v>
@@ -5893,7 +5893,7 @@
         <v>6</v>
       </c>
       <c r="B182" s="7" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C182" s="7">
         <v>2</v>
@@ -5902,7 +5902,7 @@
         <v>109</v>
       </c>
       <c r="E182" s="7" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="F182" s="7">
         <v>0</v>
@@ -5916,7 +5916,7 @@
         <v>5</v>
       </c>
       <c r="B183" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C183" s="6">
         <v>3</v>
@@ -5925,7 +5925,7 @@
         <v>6</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F183" s="6">
         <v>0</v>
@@ -5939,7 +5939,7 @@
         <v>5</v>
       </c>
       <c r="B184" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C184" s="6">
         <v>2</v>
@@ -5948,7 +5948,7 @@
         <v>7</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F184" s="6">
         <v>0</v>
@@ -5959,10 +5959,10 @@
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C185" s="2">
         <v>4</v>
@@ -5971,7 +5971,7 @@
         <v>28</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F185" s="2">
         <v>0</v>
@@ -5982,10 +5982,10 @@
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B186" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C186" s="8">
         <v>3</v>
@@ -5994,7 +5994,7 @@
         <v>188</v>
       </c>
       <c r="E186" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F186" s="8">
         <v>0</v>
@@ -6008,7 +6008,7 @@
         <v>6</v>
       </c>
       <c r="B187" s="7" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C187" s="7">
         <v>4</v>
@@ -6017,7 +6017,7 @@
         <v>17</v>
       </c>
       <c r="E187" s="7" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F187" s="7">
         <v>0</v>
@@ -6031,7 +6031,7 @@
         <v>6</v>
       </c>
       <c r="B188" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C188" s="7">
         <v>4</v>
@@ -6040,7 +6040,7 @@
         <v>23</v>
       </c>
       <c r="E188" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F188" s="7">
         <v>0</v>
@@ -6054,7 +6054,7 @@
         <v>5</v>
       </c>
       <c r="B189" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C189" s="6">
         <v>2</v>
@@ -6063,7 +6063,7 @@
         <v>3</v>
       </c>
       <c r="E189" s="6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F189" s="6">
         <v>0</v>
@@ -6074,10 +6074,10 @@
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C190" s="3">
         <v>1</v>
@@ -6086,7 +6086,7 @@
         <v>18</v>
       </c>
       <c r="E190" s="3" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F190" s="3">
         <v>0</v>
@@ -6097,10 +6097,10 @@
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C191" s="3">
         <v>3</v>
@@ -6109,7 +6109,7 @@
         <v>7</v>
       </c>
       <c r="E191" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F191" s="3">
         <v>0</v>
@@ -6120,10 +6120,10 @@
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B192" s="5" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C192" s="5">
         <v>4</v>
@@ -6132,7 +6132,7 @@
         <v>65</v>
       </c>
       <c r="E192" s="5" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="F192" s="5">
         <v>0</v>
@@ -6143,10 +6143,10 @@
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C193" s="4">
         <v>4</v>
@@ -6155,7 +6155,7 @@
         <v>29</v>
       </c>
       <c r="E193" s="4" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F193" s="4">
         <v>0</v>
@@ -6169,7 +6169,7 @@
         <v>6</v>
       </c>
       <c r="B194" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C194" s="7">
         <v>4</v>
@@ -6178,7 +6178,7 @@
         <v>59</v>
       </c>
       <c r="E194" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F194" s="7">
         <v>0</v>
@@ -6189,10 +6189,10 @@
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="C195" s="3">
         <v>3</v>
@@ -6201,7 +6201,7 @@
         <v>8</v>
       </c>
       <c r="E195" s="3" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F195" s="3">
         <v>0</v>
@@ -6212,10 +6212,10 @@
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C196" s="3">
         <v>3</v>
@@ -6224,7 +6224,7 @@
         <v>8</v>
       </c>
       <c r="E196" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F196" s="3">
         <v>0</v>
@@ -6235,10 +6235,10 @@
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C197" s="4">
         <v>3</v>
@@ -6247,7 +6247,7 @@
         <v>21</v>
       </c>
       <c r="E197" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F197" s="4">
         <v>0</v>
@@ -6261,7 +6261,7 @@
         <v>6</v>
       </c>
       <c r="B198" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C198" s="7">
         <v>3</v>
@@ -6270,7 +6270,7 @@
         <v>25</v>
       </c>
       <c r="E198" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="F198" s="7">
         <v>0</v>
@@ -6304,10 +6304,10 @@
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C200" s="3">
         <v>1</v>
@@ -6316,7 +6316,7 @@
         <v>19</v>
       </c>
       <c r="E200" s="3" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="F200" s="3">
         <v>0</v>
@@ -6327,10 +6327,10 @@
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B201" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C201" s="5">
         <v>1</v>
@@ -6339,7 +6339,7 @@
         <v>72</v>
       </c>
       <c r="E201" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F201" s="5">
         <v>0</v>
@@ -6353,7 +6353,7 @@
         <v>6</v>
       </c>
       <c r="B202" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C202" s="7">
         <v>1</v>
@@ -6362,7 +6362,7 @@
         <v>121</v>
       </c>
       <c r="E202" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="F202" s="7">
         <v>0</v>
@@ -6373,10 +6373,10 @@
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C203" s="4">
         <v>1</v>
@@ -6385,7 +6385,7 @@
         <v>66</v>
       </c>
       <c r="E203" s="4" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F203" s="4">
         <v>0</v>
@@ -6399,7 +6399,7 @@
         <v>5</v>
       </c>
       <c r="B204" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C204" s="6">
         <v>1</v>
@@ -6408,7 +6408,7 @@
         <v>12</v>
       </c>
       <c r="E204" s="6" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="F204" s="6">
         <v>0</v>
@@ -6419,10 +6419,10 @@
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B205" s="5" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C205" s="5">
         <v>4</v>
@@ -6431,7 +6431,7 @@
         <v>44</v>
       </c>
       <c r="E205" s="5" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="F205" s="5">
         <v>0</v>
@@ -6442,10 +6442,10 @@
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C206" s="4">
         <v>3</v>
@@ -6454,7 +6454,7 @@
         <v>88</v>
       </c>
       <c r="E206" s="4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F206" s="4">
         <v>0</v>
@@ -6468,7 +6468,7 @@
         <v>6</v>
       </c>
       <c r="B207" s="7" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C207" s="7">
         <v>2</v>
@@ -6477,7 +6477,7 @@
         <v>129</v>
       </c>
       <c r="E207" s="7" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="F207" s="7">
         <v>0</v>
@@ -6488,7 +6488,7 @@
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B208" s="3" t="s">
         <v>7</v>
@@ -6500,7 +6500,7 @@
         <v>9</v>
       </c>
       <c r="E208" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F208" s="3">
         <v>0</v>
@@ -6514,7 +6514,7 @@
         <v>6</v>
       </c>
       <c r="B209" s="7" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C209" s="7">
         <v>1</v>
@@ -6523,7 +6523,7 @@
         <v>101</v>
       </c>
       <c r="E209" s="7" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="F209" s="7">
         <v>1</v>
@@ -6534,10 +6534,10 @@
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="C210" s="3">
         <v>3</v>
@@ -6546,7 +6546,7 @@
         <v>9</v>
       </c>
       <c r="E210" s="3" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="F210" s="3">
         <v>0</v>
@@ -6557,10 +6557,10 @@
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C211" s="5">
         <v>4</v>
@@ -6569,7 +6569,7 @@
         <v>32</v>
       </c>
       <c r="E211" s="5" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F211" s="5">
         <v>0</v>
@@ -6583,7 +6583,7 @@
         <v>5</v>
       </c>
       <c r="B212" s="6" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C212" s="6">
         <v>3</v>
@@ -6592,7 +6592,7 @@
         <v>3</v>
       </c>
       <c r="E212" s="6" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F212" s="6">
         <v>0</v>
@@ -6606,7 +6606,7 @@
         <v>5</v>
       </c>
       <c r="B213" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C213" s="6">
         <v>4</v>
@@ -6615,7 +6615,7 @@
         <v>8</v>
       </c>
       <c r="E213" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F213" s="6">
         <v>0</v>
@@ -6626,10 +6626,10 @@
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>29</v>
+        <v>413</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C214" s="2">
         <v>4</v>
@@ -6638,7 +6638,7 @@
         <v>11</v>
       </c>
       <c r="E214" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F214" s="2">
         <v>0</v>
@@ -6649,10 +6649,10 @@
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C215" s="5">
         <v>4</v>
@@ -6661,7 +6661,7 @@
         <v>10</v>
       </c>
       <c r="E215" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F215" s="5">
         <v>0</v>
@@ -6672,10 +6672,10 @@
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C216" s="5">
         <v>2</v>
@@ -6684,7 +6684,7 @@
         <v>118</v>
       </c>
       <c r="E216" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F216" s="5">
         <v>0</v>
@@ -6695,10 +6695,10 @@
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C217" s="5">
         <v>4</v>
@@ -6707,7 +6707,7 @@
         <v>49</v>
       </c>
       <c r="E217" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F217" s="5">
         <v>0</v>
@@ -6718,10 +6718,10 @@
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C218" s="5">
         <v>3</v>
@@ -6730,7 +6730,7 @@
         <v>78</v>
       </c>
       <c r="E218" s="5" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F218" s="5">
         <v>0</v>
@@ -6741,10 +6741,10 @@
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C219" s="5">
         <v>3</v>
@@ -6753,7 +6753,7 @@
         <v>91</v>
       </c>
       <c r="E219" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F219" s="5">
         <v>0</v>
@@ -6767,7 +6767,7 @@
         <v>5</v>
       </c>
       <c r="B220" s="6" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C220" s="6">
         <v>2</v>
@@ -6776,7 +6776,7 @@
         <v>9</v>
       </c>
       <c r="E220" s="6" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F220" s="6">
         <v>0</v>
@@ -6787,10 +6787,10 @@
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
-        <v>9</v>
+        <v>414</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C221" s="8">
         <v>4</v>
@@ -6799,7 +6799,7 @@
         <v>93</v>
       </c>
       <c r="E221" s="8" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F221" s="8">
         <v>0</v>
@@ -6813,7 +6813,7 @@
         <v>6</v>
       </c>
       <c r="B222" s="7" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C222" s="7">
         <v>4</v>
@@ -6822,7 +6822,7 @@
         <v>20</v>
       </c>
       <c r="E222" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F222" s="7">
         <v>0</v>
@@ -6833,10 +6833,10 @@
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="C223" s="5">
         <v>3</v>
@@ -6845,7 +6845,7 @@
         <v>112</v>
       </c>
       <c r="E223" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="F223" s="5">
         <v>0</v>

</xml_diff>

<commit_message>
preparing for balanced exam distribution throughout week
</commit_message>
<xml_diff>
--- a/data/fall2425_course_info - Copy.xlsx
+++ b/data/fall2425_course_info - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berkercin\Desktop\Projects\Scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCFD0E4-7F4E-46BF-A40F-5B216A0069F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BED387E-C095-4997-B993-A23705E7235C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1435,7 +1435,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1E0F4194-B6AA-41D9-8C03-142586E7DC79}" name="Table2" displayName="Table2" ref="A1:G223" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:G223" xr:uid="{1E0F4194-B6AA-41D9-8C03-142586E7DC79}"/>
+  <autoFilter ref="A1:G223" xr:uid="{1E0F4194-B6AA-41D9-8C03-142586E7DC79}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="5i"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G210">
     <sortCondition ref="B1:B223"/>
   </sortState>
@@ -1748,7 +1754,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>413</v>
       </c>
@@ -1794,7 +1800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>18</v>
       </c>
@@ -1817,7 +1823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
@@ -1840,7 +1846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -1863,7 +1869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>413</v>
       </c>
@@ -1886,7 +1892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
@@ -1909,7 +1915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>413</v>
       </c>
@@ -1940,7 +1946,7 @@
         <v>407</v>
       </c>
       <c r="C10" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="5">
         <v>96</v>
@@ -1978,7 +1984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
@@ -2001,7 +2007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>18</v>
       </c>
@@ -2024,7 +2030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
@@ -2047,7 +2053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>11</v>
       </c>
@@ -2070,7 +2076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>11</v>
       </c>
@@ -2093,7 +2099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>6</v>
       </c>
@@ -2116,7 +2122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>414</v>
       </c>
@@ -2139,7 +2145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>11</v>
       </c>
@@ -2162,7 +2168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
@@ -2185,7 +2191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>414</v>
       </c>
@@ -2208,7 +2214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
@@ -2231,7 +2237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>11</v>
       </c>
@@ -2254,7 +2260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>5</v>
       </c>
@@ -2277,7 +2283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>23</v>
       </c>
@@ -2300,7 +2306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>414</v>
       </c>
@@ -2323,7 +2329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>11</v>
       </c>
@@ -2346,7 +2352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>414</v>
       </c>
@@ -2369,7 +2375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>18</v>
       </c>
@@ -2392,7 +2398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>18</v>
       </c>
@@ -2415,7 +2421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>18</v>
       </c>
@@ -2438,7 +2444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>413</v>
       </c>
@@ -2461,7 +2467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>413</v>
       </c>
@@ -2484,7 +2490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>413</v>
       </c>
@@ -2507,7 +2513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>414</v>
       </c>
@@ -2530,7 +2536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>18</v>
       </c>
@@ -2553,7 +2559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>11</v>
       </c>
@@ -2576,7 +2582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>413</v>
       </c>
@@ -2599,7 +2605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>414</v>
       </c>
@@ -2622,7 +2628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>414</v>
       </c>
@@ -2645,7 +2651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>6</v>
       </c>
@@ -2668,7 +2674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>18</v>
       </c>
@@ -2691,7 +2697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>23</v>
       </c>
@@ -2714,7 +2720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>11</v>
       </c>
@@ -2737,7 +2743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>414</v>
       </c>
@@ -2760,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>413</v>
       </c>
@@ -2783,7 +2789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>11</v>
       </c>
@@ -2806,7 +2812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>6</v>
       </c>
@@ -2829,7 +2835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>23</v>
       </c>
@@ -2852,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>414</v>
       </c>
@@ -2875,7 +2881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>414</v>
       </c>
@@ -2898,7 +2904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
         <v>414</v>
       </c>
@@ -2921,7 +2927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
         <v>414</v>
       </c>
@@ -2944,7 +2950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
         <v>414</v>
       </c>
@@ -2967,7 +2973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>414</v>
       </c>
@@ -2990,7 +2996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>414</v>
       </c>
@@ -3013,7 +3019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>414</v>
       </c>
@@ -3036,7 +3042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>414</v>
       </c>
@@ -3059,7 +3065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>23</v>
       </c>
@@ -3090,7 +3096,7 @@
         <v>407</v>
       </c>
       <c r="C60" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" s="2">
         <v>86</v>
@@ -3105,7 +3111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>413</v>
       </c>
@@ -3128,7 +3134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>23</v>
       </c>
@@ -3151,7 +3157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>413</v>
       </c>
@@ -3174,7 +3180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>18</v>
       </c>
@@ -3197,7 +3203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>6</v>
       </c>
@@ -3220,7 +3226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>23</v>
       </c>
@@ -3243,7 +3249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>23</v>
       </c>
@@ -3266,7 +3272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>6</v>
       </c>
@@ -3289,7 +3295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>11</v>
       </c>
@@ -3312,7 +3318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>23</v>
       </c>
@@ -3335,7 +3341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>413</v>
       </c>
@@ -3358,7 +3364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
         <v>414</v>
       </c>
@@ -3381,7 +3387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
         <v>414</v>
       </c>
@@ -3404,7 +3410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>413</v>
       </c>
@@ -3427,7 +3433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>18</v>
       </c>
@@ -3450,7 +3456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>413</v>
       </c>
@@ -3473,7 +3479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>413</v>
       </c>
@@ -3496,7 +3502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>413</v>
       </c>
@@ -3519,7 +3525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>6</v>
       </c>
@@ -3542,7 +3548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>11</v>
       </c>
@@ -3565,7 +3571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>23</v>
       </c>
@@ -3588,7 +3594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>23</v>
       </c>
@@ -3611,7 +3617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>18</v>
       </c>
@@ -3634,7 +3640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>23</v>
       </c>
@@ -3657,7 +3663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>23</v>
       </c>
@@ -3680,7 +3686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>23</v>
       </c>
@@ -3703,7 +3709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>23</v>
       </c>
@@ -3726,7 +3732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>23</v>
       </c>
@@ -3749,7 +3755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>23</v>
       </c>
@@ -3772,7 +3778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>23</v>
       </c>
@@ -3795,7 +3801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>23</v>
       </c>
@@ -3818,7 +3824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>23</v>
       </c>
@@ -3841,7 +3847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>23</v>
       </c>
@@ -3864,7 +3870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
         <v>6</v>
       </c>
@@ -3887,7 +3893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>11</v>
       </c>
@@ -3910,7 +3916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>6</v>
       </c>
@@ -3933,7 +3939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>11</v>
       </c>
@@ -3956,7 +3962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
         <v>6</v>
       </c>
@@ -3979,7 +3985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
         <v>414</v>
       </c>
@@ -4002,7 +4008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
         <v>6</v>
       </c>
@@ -4025,7 +4031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
         <v>414</v>
       </c>
@@ -4048,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
         <v>6</v>
       </c>
@@ -4094,7 +4100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>11</v>
       </c>
@@ -4117,7 +4123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>11</v>
       </c>
@@ -4140,7 +4146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>413</v>
       </c>
@@ -4163,7 +4169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>413</v>
       </c>
@@ -4186,7 +4192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
         <v>414</v>
       </c>
@@ -4209,7 +4215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>18</v>
       </c>
@@ -4232,7 +4238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>413</v>
       </c>
@@ -4255,7 +4261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>413</v>
       </c>
@@ -4278,7 +4284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
         <v>5</v>
       </c>
@@ -4301,7 +4307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
         <v>414</v>
       </c>
@@ -4324,7 +4330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>23</v>
       </c>
@@ -4347,7 +4353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>6</v>
       </c>
@@ -4370,7 +4376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
         <v>5</v>
       </c>
@@ -4393,7 +4399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
         <v>5</v>
       </c>
@@ -4416,7 +4422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
         <v>5</v>
       </c>
@@ -4439,7 +4445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>6</v>
       </c>
@@ -4462,7 +4468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
         <v>11</v>
       </c>
@@ -4485,7 +4491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
         <v>414</v>
       </c>
@@ -4508,7 +4514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="7" t="s">
         <v>6</v>
       </c>
@@ -4531,7 +4537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="6" t="s">
         <v>5</v>
       </c>
@@ -4554,7 +4560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>18</v>
       </c>
@@ -4577,7 +4583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="6" t="s">
         <v>5</v>
       </c>
@@ -4600,7 +4606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="7" t="s">
         <v>6</v>
       </c>
@@ -4623,7 +4629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>18</v>
       </c>
@@ -4646,7 +4652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="6" t="s">
         <v>5</v>
       </c>
@@ -4669,7 +4675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>6</v>
       </c>
@@ -4692,7 +4698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="6" t="s">
         <v>5</v>
       </c>
@@ -4715,7 +4721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
         <v>23</v>
       </c>
@@ -4738,7 +4744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
         <v>23</v>
       </c>
@@ -4761,7 +4767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
         <v>5</v>
       </c>
@@ -4784,7 +4790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>6</v>
       </c>
@@ -4807,7 +4813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>6</v>
       </c>
@@ -4830,7 +4836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
         <v>6</v>
       </c>
@@ -4853,7 +4859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
         <v>11</v>
       </c>
@@ -4876,7 +4882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>6</v>
       </c>
@@ -4899,7 +4905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
         <v>414</v>
       </c>
@@ -4922,7 +4928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="8" t="s">
         <v>414</v>
       </c>
@@ -4945,7 +4951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
         <v>11</v>
       </c>
@@ -4968,7 +4974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
         <v>23</v>
       </c>
@@ -4991,7 +4997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>6</v>
       </c>
@@ -5014,7 +5020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="8" t="s">
         <v>414</v>
       </c>
@@ -5037,7 +5043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>413</v>
       </c>
@@ -5060,7 +5066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>6</v>
       </c>
@@ -5083,7 +5089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>18</v>
       </c>
@@ -5106,7 +5112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
         <v>18</v>
       </c>
@@ -5129,7 +5135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
         <v>23</v>
       </c>
@@ -5152,7 +5158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
         <v>23</v>
       </c>
@@ -5175,7 +5181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>413</v>
       </c>
@@ -5198,7 +5204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>413</v>
       </c>
@@ -5221,7 +5227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
         <v>23</v>
       </c>
@@ -5244,7 +5250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
         <v>23</v>
       </c>
@@ -5267,7 +5273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
         <v>5</v>
       </c>
@@ -5290,7 +5296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="8" t="s">
         <v>414</v>
       </c>
@@ -5313,7 +5319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="8" t="s">
         <v>414</v>
       </c>
@@ -5336,7 +5342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
         <v>5</v>
       </c>
@@ -5359,7 +5365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="5" t="s">
         <v>11</v>
       </c>
@@ -5382,7 +5388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
         <v>6</v>
       </c>
@@ -5405,7 +5411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>413</v>
       </c>
@@ -5428,7 +5434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>413</v>
       </c>
@@ -5451,7 +5457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>413</v>
       </c>
@@ -5474,7 +5480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="5" t="s">
         <v>11</v>
       </c>
@@ -5497,7 +5503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
         <v>6</v>
       </c>
@@ -5520,7 +5526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
         <v>11</v>
       </c>
@@ -5543,7 +5549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
         <v>6</v>
       </c>
@@ -5566,7 +5572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="8" t="s">
         <v>414</v>
       </c>
@@ -5589,7 +5595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="6" t="s">
         <v>5</v>
       </c>
@@ -5612,7 +5618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>18</v>
       </c>
@@ -5635,7 +5641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>413</v>
       </c>
@@ -5658,7 +5664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="8" t="s">
         <v>414</v>
       </c>
@@ -5681,7 +5687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>18</v>
       </c>
@@ -5704,7 +5710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
         <v>414</v>
       </c>
@@ -5727,7 +5733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>413</v>
       </c>
@@ -5750,7 +5756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
         <v>414</v>
       </c>
@@ -5773,7 +5779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>413</v>
       </c>
@@ -5796,7 +5802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="8" t="s">
         <v>414</v>
       </c>
@@ -5819,7 +5825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
         <v>6</v>
       </c>
@@ -5842,7 +5848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
         <v>6</v>
       </c>
@@ -5865,7 +5871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="5" t="s">
         <v>11</v>
       </c>
@@ -5888,7 +5894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
         <v>6</v>
       </c>
@@ -5911,7 +5917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="6" t="s">
         <v>5</v>
       </c>
@@ -5934,7 +5940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="6" t="s">
         <v>5</v>
       </c>
@@ -5957,7 +5963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>413</v>
       </c>
@@ -5980,7 +5986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="8" t="s">
         <v>414</v>
       </c>
@@ -6003,7 +6009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="7" t="s">
         <v>6</v>
       </c>
@@ -6026,7 +6032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="7" t="s">
         <v>6</v>
       </c>
@@ -6049,7 +6055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
         <v>5</v>
       </c>
@@ -6072,7 +6078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
         <v>18</v>
       </c>
@@ -6095,7 +6101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
         <v>18</v>
       </c>
@@ -6118,7 +6124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="5" t="s">
         <v>11</v>
       </c>
@@ -6141,7 +6147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
         <v>23</v>
       </c>
@@ -6164,7 +6170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="7" t="s">
         <v>6</v>
       </c>
@@ -6187,7 +6193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
         <v>18</v>
       </c>
@@ -6210,7 +6216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
         <v>18</v>
       </c>
@@ -6233,7 +6239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
         <v>23</v>
       </c>
@@ -6256,7 +6262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="7" t="s">
         <v>6</v>
       </c>
@@ -6279,7 +6285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
         <v>6</v>
       </c>
@@ -6302,7 +6308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="3" t="s">
         <v>18</v>
       </c>
@@ -6325,7 +6331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="5" t="s">
         <v>11</v>
       </c>
@@ -6348,7 +6354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="7" t="s">
         <v>6</v>
       </c>
@@ -6371,7 +6377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="4" t="s">
         <v>23</v>
       </c>
@@ -6394,7 +6400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="6" t="s">
         <v>5</v>
       </c>
@@ -6417,7 +6423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="5" t="s">
         <v>11</v>
       </c>
@@ -6440,7 +6446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
         <v>23</v>
       </c>
@@ -6463,7 +6469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="7" t="s">
         <v>6</v>
       </c>
@@ -6486,7 +6492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="3" t="s">
         <v>18</v>
       </c>
@@ -6532,7 +6538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="3" t="s">
         <v>18</v>
       </c>
@@ -6555,7 +6561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="5" t="s">
         <v>11</v>
       </c>
@@ -6578,7 +6584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="6" t="s">
         <v>5</v>
       </c>
@@ -6601,7 +6607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="6" t="s">
         <v>5</v>
       </c>
@@ -6624,7 +6630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>413</v>
       </c>
@@ -6647,7 +6653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
         <v>11</v>
       </c>
@@ -6670,7 +6676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="5" t="s">
         <v>11</v>
       </c>
@@ -6693,7 +6699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="5" t="s">
         <v>11</v>
       </c>
@@ -6716,7 +6722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="5" t="s">
         <v>11</v>
       </c>
@@ -6739,7 +6745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="5" t="s">
         <v>11</v>
       </c>
@@ -6762,7 +6768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="6" t="s">
         <v>5</v>
       </c>
@@ -6785,7 +6791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
         <v>414</v>
       </c>
@@ -6808,7 +6814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="7" t="s">
         <v>6</v>
       </c>
@@ -6831,7 +6837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
written of and trying to reduce missions with cum
</commit_message>
<xml_diff>
--- a/data/fall2425_course_info - Copy.xlsx
+++ b/data/fall2425_course_info - Copy.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berkercin\Desktop\Projects\Scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BED387E-C095-4997-B993-A23705E7235C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B95906D-C8F9-4D81-BB3E-E9F5CBF95AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1435,13 +1435,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1E0F4194-B6AA-41D9-8C03-142586E7DC79}" name="Table2" displayName="Table2" ref="A1:G223" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:G223" xr:uid="{1E0F4194-B6AA-41D9-8C03-142586E7DC79}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="5i"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G223" xr:uid="{1E0F4194-B6AA-41D9-8C03-142586E7DC79}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G210">
     <sortCondition ref="B1:B223"/>
   </sortState>
@@ -1754,7 +1748,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>413</v>
       </c>
@@ -1800,7 +1794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>18</v>
       </c>
@@ -1823,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
@@ -1846,7 +1840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -1869,7 +1863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>413</v>
       </c>
@@ -1892,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
@@ -1915,7 +1909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>413</v>
       </c>
@@ -1984,7 +1978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
@@ -2007,7 +2001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>18</v>
       </c>
@@ -2030,7 +2024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
@@ -2053,7 +2047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>11</v>
       </c>
@@ -2076,7 +2070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>11</v>
       </c>
@@ -2099,7 +2093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>6</v>
       </c>
@@ -2122,7 +2116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>414</v>
       </c>
@@ -2145,7 +2139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>11</v>
       </c>
@@ -2168,7 +2162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
@@ -2191,7 +2185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>414</v>
       </c>
@@ -2214,7 +2208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
@@ -2237,7 +2231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>11</v>
       </c>
@@ -2260,7 +2254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>5</v>
       </c>
@@ -2283,7 +2277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>23</v>
       </c>
@@ -2306,7 +2300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>414</v>
       </c>
@@ -2329,7 +2323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>11</v>
       </c>
@@ -2352,7 +2346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>414</v>
       </c>
@@ -2375,7 +2369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>18</v>
       </c>
@@ -2398,7 +2392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>18</v>
       </c>
@@ -2421,7 +2415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>18</v>
       </c>
@@ -2444,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>413</v>
       </c>
@@ -2467,7 +2461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>413</v>
       </c>
@@ -2490,7 +2484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>413</v>
       </c>
@@ -2513,7 +2507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>414</v>
       </c>
@@ -2536,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>18</v>
       </c>
@@ -2559,7 +2553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>11</v>
       </c>
@@ -2582,7 +2576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>413</v>
       </c>
@@ -2605,7 +2599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>414</v>
       </c>
@@ -2628,7 +2622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>414</v>
       </c>
@@ -2651,7 +2645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>6</v>
       </c>
@@ -2674,7 +2668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>18</v>
       </c>
@@ -2697,7 +2691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>23</v>
       </c>
@@ -2720,7 +2714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>11</v>
       </c>
@@ -2743,7 +2737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>414</v>
       </c>
@@ -2766,7 +2760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>413</v>
       </c>
@@ -2789,7 +2783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>11</v>
       </c>
@@ -2812,7 +2806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>6</v>
       </c>
@@ -2835,7 +2829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>23</v>
       </c>
@@ -2858,7 +2852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>414</v>
       </c>
@@ -2881,7 +2875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>414</v>
       </c>
@@ -2904,7 +2898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
         <v>414</v>
       </c>
@@ -2927,7 +2921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
         <v>414</v>
       </c>
@@ -2950,7 +2944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
         <v>414</v>
       </c>
@@ -2973,7 +2967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>414</v>
       </c>
@@ -2996,7 +2990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>414</v>
       </c>
@@ -3019,7 +3013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>414</v>
       </c>
@@ -3042,7 +3036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>414</v>
       </c>
@@ -3065,7 +3059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>23</v>
       </c>
@@ -3111,7 +3105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>413</v>
       </c>
@@ -3134,7 +3128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>23</v>
       </c>
@@ -3157,7 +3151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>413</v>
       </c>
@@ -3180,7 +3174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>18</v>
       </c>
@@ -3203,7 +3197,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>6</v>
       </c>
@@ -3226,7 +3220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>23</v>
       </c>
@@ -3249,7 +3243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>23</v>
       </c>
@@ -3272,7 +3266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>6</v>
       </c>
@@ -3295,7 +3289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>11</v>
       </c>
@@ -3318,7 +3312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>23</v>
       </c>
@@ -3341,7 +3335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>413</v>
       </c>
@@ -3364,7 +3358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
         <v>414</v>
       </c>
@@ -3387,7 +3381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
         <v>414</v>
       </c>
@@ -3410,7 +3404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>413</v>
       </c>
@@ -3433,7 +3427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>18</v>
       </c>
@@ -3456,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>413</v>
       </c>
@@ -3479,7 +3473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>413</v>
       </c>
@@ -3502,7 +3496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>413</v>
       </c>
@@ -3525,7 +3519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>6</v>
       </c>
@@ -3548,7 +3542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>11</v>
       </c>
@@ -3571,7 +3565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>23</v>
       </c>
@@ -3594,7 +3588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>23</v>
       </c>
@@ -3617,7 +3611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>18</v>
       </c>
@@ -3640,7 +3634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>23</v>
       </c>
@@ -3663,7 +3657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>23</v>
       </c>
@@ -3686,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>23</v>
       </c>
@@ -3709,7 +3703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>23</v>
       </c>
@@ -3732,7 +3726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>23</v>
       </c>
@@ -3755,7 +3749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>23</v>
       </c>
@@ -3778,7 +3772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>23</v>
       </c>
@@ -3801,7 +3795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>23</v>
       </c>
@@ -3824,7 +3818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>23</v>
       </c>
@@ -3847,7 +3841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>23</v>
       </c>
@@ -3870,7 +3864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
         <v>6</v>
       </c>
@@ -3893,7 +3887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>11</v>
       </c>
@@ -3916,7 +3910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>6</v>
       </c>
@@ -3939,7 +3933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>11</v>
       </c>
@@ -3962,7 +3956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
         <v>6</v>
       </c>
@@ -3985,7 +3979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
         <v>414</v>
       </c>
@@ -4008,7 +4002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
         <v>6</v>
       </c>
@@ -4031,7 +4025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
         <v>414</v>
       </c>
@@ -4054,7 +4048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
         <v>6</v>
       </c>
@@ -4100,7 +4094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>11</v>
       </c>
@@ -4123,7 +4117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>11</v>
       </c>
@@ -4146,7 +4140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>413</v>
       </c>
@@ -4169,7 +4163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>413</v>
       </c>
@@ -4192,7 +4186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
         <v>414</v>
       </c>
@@ -4215,7 +4209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>18</v>
       </c>
@@ -4238,7 +4232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>413</v>
       </c>
@@ -4261,7 +4255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>413</v>
       </c>
@@ -4284,7 +4278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
         <v>5</v>
       </c>
@@ -4307,7 +4301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
         <v>414</v>
       </c>
@@ -4330,7 +4324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>23</v>
       </c>
@@ -4353,7 +4347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>6</v>
       </c>
@@ -4376,7 +4370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
         <v>5</v>
       </c>
@@ -4399,7 +4393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
         <v>5</v>
       </c>
@@ -4422,7 +4416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
         <v>5</v>
       </c>
@@ -4445,7 +4439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>6</v>
       </c>
@@ -4468,7 +4462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
         <v>11</v>
       </c>
@@ -4491,7 +4485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
         <v>414</v>
       </c>
@@ -4514,7 +4508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="7" t="s">
         <v>6</v>
       </c>
@@ -4537,7 +4531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="6" t="s">
         <v>5</v>
       </c>
@@ -4560,7 +4554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>18</v>
       </c>
@@ -4583,7 +4577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="6" t="s">
         <v>5</v>
       </c>
@@ -4606,7 +4600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="7" t="s">
         <v>6</v>
       </c>
@@ -4629,7 +4623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>18</v>
       </c>
@@ -4652,7 +4646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="6" t="s">
         <v>5</v>
       </c>
@@ -4675,7 +4669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>6</v>
       </c>
@@ -4698,7 +4692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="6" t="s">
         <v>5</v>
       </c>
@@ -4721,7 +4715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
         <v>23</v>
       </c>
@@ -4744,7 +4738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
         <v>23</v>
       </c>
@@ -4767,7 +4761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
         <v>5</v>
       </c>
@@ -4790,7 +4784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>6</v>
       </c>
@@ -4813,7 +4807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>6</v>
       </c>
@@ -4836,7 +4830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
         <v>6</v>
       </c>
@@ -4859,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
         <v>11</v>
       </c>
@@ -4882,7 +4876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>6</v>
       </c>
@@ -4905,7 +4899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
         <v>414</v>
       </c>
@@ -4928,7 +4922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="8" t="s">
         <v>414</v>
       </c>
@@ -4951,7 +4945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
         <v>11</v>
       </c>
@@ -4974,7 +4968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
         <v>23</v>
       </c>
@@ -4997,7 +4991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>6</v>
       </c>
@@ -5020,7 +5014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="8" t="s">
         <v>414</v>
       </c>
@@ -5043,7 +5037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>413</v>
       </c>
@@ -5066,7 +5060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>6</v>
       </c>
@@ -5089,7 +5083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>18</v>
       </c>
@@ -5112,7 +5106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
         <v>18</v>
       </c>
@@ -5135,7 +5129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
         <v>23</v>
       </c>
@@ -5158,7 +5152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
         <v>23</v>
       </c>
@@ -5181,7 +5175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>413</v>
       </c>
@@ -5204,7 +5198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>413</v>
       </c>
@@ -5227,7 +5221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
         <v>23</v>
       </c>
@@ -5250,7 +5244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
         <v>23</v>
       </c>
@@ -5273,7 +5267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
         <v>5</v>
       </c>
@@ -5296,7 +5290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="8" t="s">
         <v>414</v>
       </c>
@@ -5319,7 +5313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="8" t="s">
         <v>414</v>
       </c>
@@ -5342,7 +5336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
         <v>5</v>
       </c>
@@ -5365,7 +5359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="5" t="s">
         <v>11</v>
       </c>
@@ -5388,7 +5382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
         <v>6</v>
       </c>
@@ -5411,7 +5405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>413</v>
       </c>
@@ -5434,7 +5428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>413</v>
       </c>
@@ -5457,7 +5451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>413</v>
       </c>
@@ -5480,7 +5474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="5" t="s">
         <v>11</v>
       </c>
@@ -5503,7 +5497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
         <v>6</v>
       </c>
@@ -5526,7 +5520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
         <v>11</v>
       </c>
@@ -5549,7 +5543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
         <v>6</v>
       </c>
@@ -5572,7 +5566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="8" t="s">
         <v>414</v>
       </c>
@@ -5595,7 +5589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="6" t="s">
         <v>5</v>
       </c>
@@ -5618,7 +5612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>18</v>
       </c>
@@ -5641,7 +5635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>413</v>
       </c>
@@ -5664,7 +5658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="8" t="s">
         <v>414</v>
       </c>
@@ -5687,7 +5681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>18</v>
       </c>
@@ -5710,7 +5704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
         <v>414</v>
       </c>
@@ -5733,7 +5727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>413</v>
       </c>
@@ -5756,7 +5750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
         <v>414</v>
       </c>
@@ -5779,7 +5773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>413</v>
       </c>
@@ -5802,7 +5796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="8" t="s">
         <v>414</v>
       </c>
@@ -5825,7 +5819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
         <v>6</v>
       </c>
@@ -5848,7 +5842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
         <v>6</v>
       </c>
@@ -5871,7 +5865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="5" t="s">
         <v>11</v>
       </c>
@@ -5894,7 +5888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
         <v>6</v>
       </c>
@@ -5917,7 +5911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="6" t="s">
         <v>5</v>
       </c>
@@ -5940,7 +5934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="6" t="s">
         <v>5</v>
       </c>
@@ -5963,7 +5957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>413</v>
       </c>
@@ -5986,7 +5980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="8" t="s">
         <v>414</v>
       </c>
@@ -6009,7 +6003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="7" t="s">
         <v>6</v>
       </c>
@@ -6032,7 +6026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="7" t="s">
         <v>6</v>
       </c>
@@ -6055,7 +6049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
         <v>5</v>
       </c>
@@ -6078,7 +6072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
         <v>18</v>
       </c>
@@ -6101,7 +6095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
         <v>18</v>
       </c>
@@ -6124,7 +6118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="5" t="s">
         <v>11</v>
       </c>
@@ -6147,7 +6141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
         <v>23</v>
       </c>
@@ -6170,7 +6164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="7" t="s">
         <v>6</v>
       </c>
@@ -6193,7 +6187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
         <v>18</v>
       </c>
@@ -6216,7 +6210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
         <v>18</v>
       </c>
@@ -6239,7 +6233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
         <v>23</v>
       </c>
@@ -6262,7 +6256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="7" t="s">
         <v>6</v>
       </c>
@@ -6285,7 +6279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
         <v>6</v>
       </c>
@@ -6308,7 +6302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="3" t="s">
         <v>18</v>
       </c>
@@ -6331,7 +6325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="5" t="s">
         <v>11</v>
       </c>
@@ -6354,7 +6348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="7" t="s">
         <v>6</v>
       </c>
@@ -6377,7 +6371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="4" t="s">
         <v>23</v>
       </c>
@@ -6400,7 +6394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="6" t="s">
         <v>5</v>
       </c>
@@ -6423,7 +6417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="5" t="s">
         <v>11</v>
       </c>
@@ -6446,7 +6440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
         <v>23</v>
       </c>
@@ -6469,7 +6463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="7" t="s">
         <v>6</v>
       </c>
@@ -6492,7 +6486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="3" t="s">
         <v>18</v>
       </c>
@@ -6538,7 +6532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="3" t="s">
         <v>18</v>
       </c>
@@ -6561,7 +6555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="5" t="s">
         <v>11</v>
       </c>
@@ -6584,7 +6578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" s="6" t="s">
         <v>5</v>
       </c>
@@ -6607,7 +6601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" s="6" t="s">
         <v>5</v>
       </c>
@@ -6630,7 +6624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>413</v>
       </c>
@@ -6653,7 +6647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
         <v>11</v>
       </c>
@@ -6676,7 +6670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="5" t="s">
         <v>11</v>
       </c>
@@ -6699,7 +6693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="5" t="s">
         <v>11</v>
       </c>
@@ -6722,7 +6716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="5" t="s">
         <v>11</v>
       </c>
@@ -6745,7 +6739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="5" t="s">
         <v>11</v>
       </c>
@@ -6768,7 +6762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="6" t="s">
         <v>5</v>
       </c>
@@ -6791,7 +6785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
         <v>414</v>
       </c>
@@ -6814,7 +6808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" s="7" t="s">
         <v>6</v>
       </c>
@@ -6837,7 +6831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="5" t="s">
         <v>11</v>
       </c>

</xml_diff>